<commit_message>
fix: PDF뷰어 6.0 분기/7.0 시드 risk_tag(network) 보정 → high 승격, 미리보기 재캡처
</commit_message>
<xml_diff>
--- a/outputs/sheets/goodnotes.xlsx
+++ b/outputs/sheets/goodnotes.xlsx
@@ -1215,7 +1215,7 @@
       </c>
       <c r="C9" s="3" t="inlineStr">
         <is>
-          <t>mid</t>
+          <t>high</t>
         </is>
       </c>
       <c r="D9" s="8" t="inlineStr"/>
@@ -1243,7 +1243,7 @@
       </c>
       <c r="C10" s="3" t="inlineStr">
         <is>
-          <t>mid</t>
+          <t>high</t>
         </is>
       </c>
       <c r="D10" s="8" t="inlineStr"/>
@@ -1271,7 +1271,7 @@
       </c>
       <c r="C11" s="3" t="inlineStr">
         <is>
-          <t>mid</t>
+          <t>high</t>
         </is>
       </c>
       <c r="D11" s="8" t="inlineStr"/>
@@ -1299,7 +1299,7 @@
       </c>
       <c r="C12" s="3" t="inlineStr">
         <is>
-          <t>mid</t>
+          <t>high</t>
         </is>
       </c>
       <c r="D12" s="8" t="inlineStr"/>
@@ -1327,7 +1327,7 @@
       </c>
       <c r="C13" s="3" t="inlineStr">
         <is>
-          <t>low</t>
+          <t>high</t>
         </is>
       </c>
       <c r="D13" s="8" t="inlineStr"/>

</xml_diff>